<commit_message>
fix(ui): align dashboard button across banking and card pages
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/overseas-payment/WeCMS_Overseas_Payment_download_EN.xlsx
+++ b/src/main/resources/templates/overseas-payment/WeCMS_Overseas_Payment_download_EN.xlsx
@@ -1054,23 +1054,23 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="22.1809523809524" customWidth="1"/>
-    <col min="3" max="3" width="16.0857142857143" customWidth="1"/>
-    <col min="4" max="6" width="20.5428571428571" customWidth="1"/>
-    <col min="7" max="7" width="24.6285714285714" customWidth="1"/>
-    <col min="8" max="8" width="26.8190476190476" customWidth="1"/>
-    <col min="9" max="10" width="29.0857142857143" customWidth="1"/>
-    <col min="11" max="11" width="34.3619047619048" customWidth="1"/>
-    <col min="12" max="12" width="25.8190476190476" customWidth="1"/>
-    <col min="13" max="13" width="23.9047619047619" customWidth="1"/>
-    <col min="14" max="14" width="23.1809523809524" customWidth="1"/>
-    <col min="15" max="16" width="26.4571428571429" customWidth="1"/>
-    <col min="17" max="17" width="31.4571428571429" customWidth="1"/>
-    <col min="18" max="22" width="22.1809523809524" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="20.0"/>
+    <col min="2" max="2" customWidth="true" width="22.1809523809524"/>
+    <col min="3" max="3" customWidth="true" width="16.0857142857143"/>
+    <col min="4" max="6" customWidth="true" width="20.5428571428571"/>
+    <col min="7" max="7" customWidth="true" width="24.6285714285714"/>
+    <col min="8" max="8" customWidth="true" width="26.8190476190476"/>
+    <col min="9" max="10" customWidth="true" width="29.0857142857143"/>
+    <col min="11" max="11" customWidth="true" width="34.3619047619048"/>
+    <col min="12" max="12" customWidth="true" width="25.8190476190476"/>
+    <col min="13" max="13" customWidth="true" width="23.9047619047619"/>
+    <col min="14" max="14" customWidth="true" width="23.1809523809524"/>
+    <col min="15" max="16" customWidth="true" width="26.4571428571429"/>
+    <col min="17" max="17" customWidth="true" width="31.4571428571429"/>
+    <col min="18" max="22" customWidth="true" width="22.1809523809524"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.5" customHeight="1" spans="1:22">
@@ -1238,868 +1238,6 @@
       <c r="U5" s="5"/>
       <c r="V5" s="5"/>
     </row>
-    <row r="6" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-    </row>
-    <row r="7" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="5"/>
-      <c r="T7" s="5"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5"/>
-    </row>
-    <row r="8" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="5"/>
-      <c r="T8" s="5"/>
-      <c r="U8" s="5"/>
-      <c r="V8" s="5"/>
-    </row>
-    <row r="9" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="5"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="5"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="5"/>
-    </row>
-    <row r="10" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-      <c r="Q10" s="5"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="5"/>
-      <c r="T10" s="5"/>
-      <c r="U10" s="5"/>
-      <c r="V10" s="5"/>
-    </row>
-    <row r="11" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="5"/>
-      <c r="P11" s="5"/>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
-      <c r="T11" s="5"/>
-      <c r="U11" s="5"/>
-      <c r="V11" s="5"/>
-    </row>
-    <row r="12" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="5"/>
-      <c r="P12" s="5"/>
-      <c r="Q12" s="5"/>
-      <c r="R12" s="5"/>
-      <c r="S12" s="5"/>
-      <c r="T12" s="5"/>
-      <c r="U12" s="5"/>
-      <c r="V12" s="5"/>
-    </row>
-    <row r="13" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="5"/>
-      <c r="P13" s="5"/>
-      <c r="Q13" s="5"/>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
-      <c r="V13" s="5"/>
-    </row>
-    <row r="14" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="5"/>
-      <c r="R14" s="5"/>
-      <c r="S14" s="5"/>
-      <c r="T14" s="5"/>
-      <c r="U14" s="5"/>
-      <c r="V14" s="5"/>
-    </row>
-    <row r="15" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="5"/>
-      <c r="P15" s="5"/>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5"/>
-      <c r="S15" s="5"/>
-      <c r="T15" s="5"/>
-      <c r="U15" s="5"/>
-      <c r="V15" s="5"/>
-    </row>
-    <row r="16" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-      <c r="L16" s="5"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="5"/>
-      <c r="P16" s="5"/>
-      <c r="Q16" s="5"/>
-      <c r="R16" s="5"/>
-      <c r="S16" s="5"/>
-      <c r="T16" s="5"/>
-      <c r="U16" s="5"/>
-      <c r="V16" s="5"/>
-    </row>
-    <row r="17" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-      <c r="R17" s="5"/>
-      <c r="S17" s="5"/>
-      <c r="T17" s="5"/>
-      <c r="U17" s="5"/>
-      <c r="V17" s="5"/>
-    </row>
-    <row r="18" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-      <c r="R18" s="5"/>
-      <c r="S18" s="5"/>
-      <c r="T18" s="5"/>
-      <c r="U18" s="5"/>
-      <c r="V18" s="5"/>
-    </row>
-    <row r="19" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
-      <c r="U19" s="5"/>
-      <c r="V19" s="5"/>
-    </row>
-    <row r="20" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
-      <c r="U20" s="5"/>
-      <c r="V20" s="5"/>
-    </row>
-    <row r="21" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="5"/>
-      <c r="S21" s="5"/>
-      <c r="T21" s="5"/>
-      <c r="U21" s="5"/>
-      <c r="V21" s="5"/>
-    </row>
-    <row r="22" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="5"/>
-      <c r="V22" s="5"/>
-    </row>
-    <row r="23" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="6"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-    </row>
-    <row r="24" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="6"/>
-      <c r="O24" s="5"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5"/>
-      <c r="S24" s="5"/>
-      <c r="T24" s="5"/>
-      <c r="U24" s="5"/>
-      <c r="V24" s="5"/>
-    </row>
-    <row r="25" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-      <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
-      <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="6"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5"/>
-      <c r="S25" s="5"/>
-      <c r="T25" s="5"/>
-      <c r="U25" s="5"/>
-      <c r="V25" s="5"/>
-    </row>
-    <row r="26" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="5"/>
-      <c r="S26" s="5"/>
-      <c r="T26" s="5"/>
-      <c r="U26" s="5"/>
-      <c r="V26" s="5"/>
-    </row>
-    <row r="27" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="8"/>
-      <c r="R27" s="5"/>
-      <c r="S27" s="5"/>
-      <c r="T27" s="5"/>
-      <c r="U27" s="5"/>
-      <c r="V27" s="5"/>
-    </row>
-    <row r="28" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="6"/>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
-      <c r="U28" s="5"/>
-      <c r="V28" s="5"/>
-    </row>
-    <row r="29" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="5"/>
-    </row>
-    <row r="30" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
-      <c r="S30" s="5"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
-      <c r="V30" s="5"/>
-    </row>
-    <row r="31" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="8"/>
-      <c r="R31" s="5"/>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
-      <c r="U31" s="5"/>
-      <c r="V31" s="5"/>
-    </row>
-    <row r="32" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5"/>
-      <c r="R32" s="5"/>
-      <c r="S32" s="5"/>
-      <c r="T32" s="5"/>
-      <c r="U32" s="5"/>
-      <c r="V32" s="5"/>
-    </row>
-    <row r="33" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
-      <c r="L33" s="5"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="5"/>
-      <c r="P33" s="5"/>
-      <c r="Q33" s="5"/>
-      <c r="R33" s="5"/>
-      <c r="S33" s="5"/>
-      <c r="T33" s="5"/>
-      <c r="U33" s="5"/>
-      <c r="V33" s="5"/>
-    </row>
-    <row r="34" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A34" s="5"/>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
-      <c r="L34" s="5"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="6"/>
-      <c r="O34" s="5"/>
-      <c r="P34" s="5"/>
-      <c r="Q34" s="5"/>
-      <c r="R34" s="5"/>
-      <c r="S34" s="5"/>
-      <c r="T34" s="5"/>
-      <c r="U34" s="5"/>
-      <c r="V34" s="5"/>
-    </row>
-    <row r="35" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="6"/>
-      <c r="O35" s="5"/>
-      <c r="P35" s="5"/>
-      <c r="Q35" s="5"/>
-      <c r="R35" s="5"/>
-      <c r="S35" s="5"/>
-      <c r="T35" s="5"/>
-      <c r="U35" s="5"/>
-      <c r="V35" s="5"/>
-    </row>
-    <row r="36" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A36" s="5"/>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="5"/>
-      <c r="P36" s="5"/>
-      <c r="Q36" s="5"/>
-      <c r="R36" s="5"/>
-      <c r="S36" s="5"/>
-      <c r="T36" s="5"/>
-      <c r="U36" s="5"/>
-      <c r="V36" s="5"/>
-    </row>
-    <row r="37" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A37" s="5"/>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-      <c r="L37" s="5"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="5"/>
-      <c r="P37" s="5"/>
-      <c r="Q37" s="5"/>
-      <c r="R37" s="5"/>
-      <c r="S37" s="5"/>
-      <c r="T37" s="5"/>
-      <c r="U37" s="5"/>
-      <c r="V37" s="5"/>
-    </row>
-    <row r="38" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A38" s="5"/>
-      <c r="B38" s="5"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
-      <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
-      <c r="L38" s="5"/>
-      <c r="M38" s="5"/>
-      <c r="N38" s="6"/>
-      <c r="O38" s="5"/>
-      <c r="P38" s="5"/>
-      <c r="Q38" s="5"/>
-      <c r="R38" s="5"/>
-      <c r="S38" s="5"/>
-      <c r="T38" s="5"/>
-      <c r="U38" s="5"/>
-      <c r="V38" s="5"/>
-    </row>
-    <row r="39" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5"/>
-      <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
-      <c r="L39" s="5"/>
-      <c r="M39" s="5"/>
-      <c r="N39" s="6"/>
-      <c r="O39" s="5"/>
-      <c r="P39" s="5"/>
-      <c r="Q39" s="5"/>
-      <c r="R39" s="5"/>
-      <c r="S39" s="5"/>
-      <c r="T39" s="5"/>
-      <c r="U39" s="5"/>
-      <c r="V39" s="5"/>
-    </row>
-    <row r="40" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="5"/>
-      <c r="N40" s="6"/>
-      <c r="O40" s="5"/>
-      <c r="P40" s="5"/>
-      <c r="Q40" s="5"/>
-      <c r="R40" s="5"/>
-      <c r="S40" s="5"/>
-      <c r="T40" s="5"/>
-      <c r="U40" s="5"/>
-      <c r="V40" s="5"/>
-    </row>
-    <row r="41" ht="16.5" customHeight="1" spans="1:22">
-      <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
-      <c r="L41" s="5"/>
-      <c r="M41" s="5"/>
-      <c r="N41" s="6"/>
-      <c r="O41" s="5"/>
-      <c r="P41" s="5"/>
-      <c r="Q41" s="5"/>
-      <c r="R41" s="5"/>
-      <c r="S41" s="5"/>
-      <c r="T41" s="5"/>
-      <c r="U41" s="5"/>
-      <c r="V41" s="5"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:T3"/>

</xml_diff>